<commit_message>
Apply modal workbook layout reference
</commit_message>
<xml_diff>
--- a/Studymaterials/中学生英作文助動詞can編.xlsx
+++ b/Studymaterials/中学生英作文助動詞can編.xlsx
@@ -1075,12 +1075,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:J191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
-    <col width="13" customWidth="1" style="6" min="1" max="1"/>
+    <col width="9.6328125" customWidth="1" style="6" min="1" max="1"/>
     <col width="13" customWidth="1" style="6" min="2" max="2"/>
     <col width="13" customWidth="1" style="6" min="3" max="3"/>
     <col width="13" customWidth="1" style="6" min="4" max="4"/>
@@ -1170,7 +1170,7 @@
       <c r="I5" s="27" t="n"/>
       <c r="J5" s="57" t="n"/>
     </row>
-    <row r="6" ht="20" customHeight="1" s="6">
+    <row r="6" ht="18" customHeight="1" s="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -1186,7 +1186,7 @@
       <c r="I6" s="27" t="n"/>
       <c r="J6" s="57" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1" s="6">
+    <row r="7" ht="18" customHeight="1" s="6">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -1218,7 +1218,7 @@
       <c r="I8" s="27" t="n"/>
       <c r="J8" s="57" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1" s="6">
+    <row r="9" ht="18" customHeight="1" s="6">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -1234,7 +1234,7 @@
       <c r="I9" s="27" t="n"/>
       <c r="J9" s="57" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1" s="6">
+    <row r="10" ht="18" customHeight="1" s="6">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -1250,7 +1250,7 @@
       <c r="I10" s="27" t="n"/>
       <c r="J10" s="57" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1" s="6">
+    <row r="11" ht="18" customHeight="1" s="6">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -1282,7 +1282,7 @@
       <c r="I12" s="27" t="n"/>
       <c r="J12" s="57" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1" s="6">
+    <row r="13" ht="18" customHeight="1" s="6">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -1298,7 +1298,7 @@
       <c r="I13" s="27" t="n"/>
       <c r="J13" s="57" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1" s="6">
+    <row r="14" ht="18" customHeight="1" s="6">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -1330,7 +1330,7 @@
       <c r="I15" s="27" t="n"/>
       <c r="J15" s="57" t="n"/>
     </row>
-    <row r="16" ht="20" customHeight="1" s="6">
+    <row r="16" ht="18" customHeight="1" s="6">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -1346,7 +1346,7 @@
       <c r="I16" s="27" t="n"/>
       <c r="J16" s="57" t="n"/>
     </row>
-    <row r="17" ht="20" customHeight="1" s="6">
+    <row r="17" ht="18" customHeight="1" s="6">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -1378,7 +1378,7 @@
       <c r="I18" s="27" t="n"/>
       <c r="J18" s="57" t="n"/>
     </row>
-    <row r="19" ht="20" customHeight="1" s="6">
+    <row r="19" ht="18" customHeight="1" s="6">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -1394,7 +1394,7 @@
       <c r="I19" s="27" t="n"/>
       <c r="J19" s="57" t="n"/>
     </row>
-    <row r="20" ht="20" customHeight="1" s="6">
+    <row r="20" ht="18" customHeight="1" s="6">
       <c r="A20" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -1410,7 +1410,7 @@
       <c r="I20" s="27" t="n"/>
       <c r="J20" s="57" t="n"/>
     </row>
-    <row r="21" ht="20" customHeight="1" s="6">
+    <row r="21" ht="18" customHeight="1" s="6">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -1426,7 +1426,7 @@
       <c r="I21" s="27" t="n"/>
       <c r="J21" s="57" t="n"/>
     </row>
-    <row r="22" ht="20" customHeight="1" s="6">
+    <row r="22" ht="18" customHeight="1" s="6">
       <c r="A22" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -1503,7 +1503,7 @@
       <c r="I26" s="27" t="n"/>
       <c r="J26" s="57" t="n"/>
     </row>
-    <row r="27" ht="20" customHeight="1" s="6">
+    <row r="27" ht="18" customHeight="1" s="6">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -1519,7 +1519,7 @@
       <c r="I27" s="27" t="n"/>
       <c r="J27" s="57" t="n"/>
     </row>
-    <row r="28" ht="20" customHeight="1" s="6">
+    <row r="28" ht="18" customHeight="1" s="6">
       <c r="A28" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -1551,7 +1551,7 @@
       <c r="I29" s="27" t="n"/>
       <c r="J29" s="57" t="n"/>
     </row>
-    <row r="30" ht="20" customHeight="1" s="6">
+    <row r="30" ht="18" customHeight="1" s="6">
       <c r="A30" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -1567,7 +1567,7 @@
       <c r="I30" s="27" t="n"/>
       <c r="J30" s="57" t="n"/>
     </row>
-    <row r="31" ht="20" customHeight="1" s="6">
+    <row r="31" ht="18" customHeight="1" s="6">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -1583,7 +1583,7 @@
       <c r="I31" s="27" t="n"/>
       <c r="J31" s="57" t="n"/>
     </row>
-    <row r="32" ht="20" customHeight="1" s="6">
+    <row r="32" ht="18" customHeight="1" s="6">
       <c r="A32" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -1615,7 +1615,7 @@
       <c r="I33" s="27" t="n"/>
       <c r="J33" s="57" t="n"/>
     </row>
-    <row r="34" ht="20" customHeight="1" s="6">
+    <row r="34" ht="18" customHeight="1" s="6">
       <c r="A34" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -1631,7 +1631,7 @@
       <c r="I34" s="27" t="n"/>
       <c r="J34" s="57" t="n"/>
     </row>
-    <row r="35" ht="20" customHeight="1" s="6">
+    <row r="35" ht="18" customHeight="1" s="6">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -1663,7 +1663,7 @@
       <c r="I36" s="27" t="n"/>
       <c r="J36" s="57" t="n"/>
     </row>
-    <row r="37" ht="20" customHeight="1" s="6">
+    <row r="37" ht="18" customHeight="1" s="6">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -1679,7 +1679,7 @@
       <c r="I37" s="27" t="n"/>
       <c r="J37" s="57" t="n"/>
     </row>
-    <row r="38" ht="20" customHeight="1" s="6">
+    <row r="38" ht="18" customHeight="1" s="6">
       <c r="A38" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -1711,7 +1711,7 @@
       <c r="I39" s="27" t="n"/>
       <c r="J39" s="57" t="n"/>
     </row>
-    <row r="40" ht="20" customHeight="1" s="6">
+    <row r="40" ht="18" customHeight="1" s="6">
       <c r="A40" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -1727,7 +1727,7 @@
       <c r="I40" s="27" t="n"/>
       <c r="J40" s="57" t="n"/>
     </row>
-    <row r="41" ht="20" customHeight="1" s="6">
+    <row r="41" ht="18" customHeight="1" s="6">
       <c r="A41" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -1743,7 +1743,7 @@
       <c r="I41" s="27" t="n"/>
       <c r="J41" s="57" t="n"/>
     </row>
-    <row r="42" ht="20" customHeight="1" s="6">
+    <row r="42" ht="18" customHeight="1" s="6">
       <c r="A42" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -1759,7 +1759,7 @@
       <c r="I42" s="27" t="n"/>
       <c r="J42" s="57" t="n"/>
     </row>
-    <row r="43" ht="20" customHeight="1" s="6">
+    <row r="43" ht="18" customHeight="1" s="6">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -1836,7 +1836,7 @@
       <c r="I47" s="27" t="n"/>
       <c r="J47" s="57" t="n"/>
     </row>
-    <row r="48" ht="20" customHeight="1" s="6">
+    <row r="48" ht="18" customHeight="1" s="6">
       <c r="A48" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -1852,7 +1852,7 @@
       <c r="I48" s="27" t="n"/>
       <c r="J48" s="57" t="n"/>
     </row>
-    <row r="49" ht="20" customHeight="1" s="6">
+    <row r="49" ht="18" customHeight="1" s="6">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -1884,7 +1884,7 @@
       <c r="I50" s="27" t="n"/>
       <c r="J50" s="57" t="n"/>
     </row>
-    <row r="51" ht="20" customHeight="1" s="6">
+    <row r="51" ht="18" customHeight="1" s="6">
       <c r="A51" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -1900,7 +1900,7 @@
       <c r="I51" s="27" t="n"/>
       <c r="J51" s="57" t="n"/>
     </row>
-    <row r="52" ht="20" customHeight="1" s="6">
+    <row r="52" ht="18" customHeight="1" s="6">
       <c r="A52" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -1916,7 +1916,7 @@
       <c r="I52" s="27" t="n"/>
       <c r="J52" s="57" t="n"/>
     </row>
-    <row r="53" ht="20" customHeight="1" s="6">
+    <row r="53" ht="18" customHeight="1" s="6">
       <c r="A53" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -1948,7 +1948,7 @@
       <c r="I54" s="27" t="n"/>
       <c r="J54" s="57" t="n"/>
     </row>
-    <row r="55" ht="20" customHeight="1" s="6">
+    <row r="55" ht="18" customHeight="1" s="6">
       <c r="A55" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -1964,7 +1964,7 @@
       <c r="I55" s="27" t="n"/>
       <c r="J55" s="57" t="n"/>
     </row>
-    <row r="56" ht="20" customHeight="1" s="6">
+    <row r="56" ht="18" customHeight="1" s="6">
       <c r="A56" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -1996,7 +1996,7 @@
       <c r="I57" s="27" t="n"/>
       <c r="J57" s="57" t="n"/>
     </row>
-    <row r="58" ht="20" customHeight="1" s="6">
+    <row r="58" ht="18" customHeight="1" s="6">
       <c r="A58" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -2012,7 +2012,7 @@
       <c r="I58" s="27" t="n"/>
       <c r="J58" s="57" t="n"/>
     </row>
-    <row r="59" ht="20" customHeight="1" s="6">
+    <row r="59" ht="18" customHeight="1" s="6">
       <c r="A59" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -2044,7 +2044,7 @@
       <c r="I60" s="27" t="n"/>
       <c r="J60" s="57" t="n"/>
     </row>
-    <row r="61" ht="20" customHeight="1" s="6">
+    <row r="61" ht="18" customHeight="1" s="6">
       <c r="A61" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -2060,7 +2060,7 @@
       <c r="I61" s="27" t="n"/>
       <c r="J61" s="57" t="n"/>
     </row>
-    <row r="62" ht="20" customHeight="1" s="6">
+    <row r="62" ht="18" customHeight="1" s="6">
       <c r="A62" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -2076,7 +2076,7 @@
       <c r="I62" s="27" t="n"/>
       <c r="J62" s="57" t="n"/>
     </row>
-    <row r="63" ht="20" customHeight="1" s="6">
+    <row r="63" ht="18" customHeight="1" s="6">
       <c r="A63" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -2092,7 +2092,7 @@
       <c r="I63" s="27" t="n"/>
       <c r="J63" s="57" t="n"/>
     </row>
-    <row r="64" ht="20" customHeight="1" s="6">
+    <row r="64" ht="18" customHeight="1" s="6">
       <c r="A64" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -2169,7 +2169,7 @@
       <c r="I68" s="27" t="n"/>
       <c r="J68" s="57" t="n"/>
     </row>
-    <row r="69" ht="20" customHeight="1" s="6">
+    <row r="69" ht="18" customHeight="1" s="6">
       <c r="A69" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -2185,7 +2185,7 @@
       <c r="I69" s="27" t="n"/>
       <c r="J69" s="57" t="n"/>
     </row>
-    <row r="70" ht="20" customHeight="1" s="6">
+    <row r="70" ht="18" customHeight="1" s="6">
       <c r="A70" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -2217,7 +2217,7 @@
       <c r="I71" s="27" t="n"/>
       <c r="J71" s="57" t="n"/>
     </row>
-    <row r="72" ht="20" customHeight="1" s="6">
+    <row r="72" ht="18" customHeight="1" s="6">
       <c r="A72" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -2233,7 +2233,7 @@
       <c r="I72" s="27" t="n"/>
       <c r="J72" s="57" t="n"/>
     </row>
-    <row r="73" ht="20" customHeight="1" s="6">
+    <row r="73" ht="18" customHeight="1" s="6">
       <c r="A73" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -2249,7 +2249,7 @@
       <c r="I73" s="27" t="n"/>
       <c r="J73" s="57" t="n"/>
     </row>
-    <row r="74" ht="20" customHeight="1" s="6">
+    <row r="74" ht="18" customHeight="1" s="6">
       <c r="A74" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -2281,7 +2281,7 @@
       <c r="I75" s="27" t="n"/>
       <c r="J75" s="57" t="n"/>
     </row>
-    <row r="76" ht="20" customHeight="1" s="6">
+    <row r="76" ht="18" customHeight="1" s="6">
       <c r="A76" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -2297,7 +2297,7 @@
       <c r="I76" s="27" t="n"/>
       <c r="J76" s="57" t="n"/>
     </row>
-    <row r="77" ht="20" customHeight="1" s="6">
+    <row r="77" ht="18" customHeight="1" s="6">
       <c r="A77" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -2329,7 +2329,7 @@
       <c r="I78" s="27" t="n"/>
       <c r="J78" s="57" t="n"/>
     </row>
-    <row r="79" ht="20" customHeight="1" s="6">
+    <row r="79" ht="18" customHeight="1" s="6">
       <c r="A79" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -2345,7 +2345,7 @@
       <c r="I79" s="27" t="n"/>
       <c r="J79" s="57" t="n"/>
     </row>
-    <row r="80" ht="20" customHeight="1" s="6">
+    <row r="80" ht="18" customHeight="1" s="6">
       <c r="A80" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -2377,7 +2377,7 @@
       <c r="I81" s="27" t="n"/>
       <c r="J81" s="57" t="n"/>
     </row>
-    <row r="82" ht="20" customHeight="1" s="6">
+    <row r="82" ht="18" customHeight="1" s="6">
       <c r="A82" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -2393,7 +2393,7 @@
       <c r="I82" s="27" t="n"/>
       <c r="J82" s="57" t="n"/>
     </row>
-    <row r="83" ht="20" customHeight="1" s="6">
+    <row r="83" ht="18" customHeight="1" s="6">
       <c r="A83" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -2409,7 +2409,7 @@
       <c r="I83" s="27" t="n"/>
       <c r="J83" s="57" t="n"/>
     </row>
-    <row r="84" ht="20" customHeight="1" s="6">
+    <row r="84" ht="18" customHeight="1" s="6">
       <c r="A84" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -2425,7 +2425,7 @@
       <c r="I84" s="27" t="n"/>
       <c r="J84" s="57" t="n"/>
     </row>
-    <row r="85" ht="20" customHeight="1" s="6">
+    <row r="85" ht="18" customHeight="1" s="6">
       <c r="A85" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -2503,7 +2503,7 @@
       <c r="I89" s="27" t="n"/>
       <c r="J89" s="57" t="n"/>
     </row>
-    <row r="90" ht="20" customHeight="1" s="6">
+    <row r="90" ht="18" customHeight="1" s="6">
       <c r="A90" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -2519,7 +2519,7 @@
       <c r="I90" s="27" t="n"/>
       <c r="J90" s="57" t="n"/>
     </row>
-    <row r="91" ht="20" customHeight="1" s="6">
+    <row r="91" ht="18" customHeight="1" s="6">
       <c r="A91" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -2551,7 +2551,7 @@
       <c r="I92" s="27" t="n"/>
       <c r="J92" s="57" t="n"/>
     </row>
-    <row r="93" ht="20" customHeight="1" s="6">
+    <row r="93" ht="18" customHeight="1" s="6">
       <c r="A93" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -2567,7 +2567,7 @@
       <c r="I93" s="27" t="n"/>
       <c r="J93" s="57" t="n"/>
     </row>
-    <row r="94" ht="20" customHeight="1" s="6">
+    <row r="94" ht="18" customHeight="1" s="6">
       <c r="A94" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -2583,7 +2583,7 @@
       <c r="I94" s="27" t="n"/>
       <c r="J94" s="57" t="n"/>
     </row>
-    <row r="95" ht="20" customHeight="1" s="6">
+    <row r="95" ht="18" customHeight="1" s="6">
       <c r="A95" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -2615,7 +2615,7 @@
       <c r="I96" s="27" t="n"/>
       <c r="J96" s="57" t="n"/>
     </row>
-    <row r="97" ht="20" customHeight="1" s="6">
+    <row r="97" ht="18" customHeight="1" s="6">
       <c r="A97" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -2631,7 +2631,7 @@
       <c r="I97" s="27" t="n"/>
       <c r="J97" s="57" t="n"/>
     </row>
-    <row r="98" ht="20" customHeight="1" s="6">
+    <row r="98" ht="18" customHeight="1" s="6">
       <c r="A98" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -2663,7 +2663,7 @@
       <c r="I99" s="27" t="n"/>
       <c r="J99" s="57" t="n"/>
     </row>
-    <row r="100" ht="20" customHeight="1" s="6">
+    <row r="100" ht="18" customHeight="1" s="6">
       <c r="A100" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -2679,7 +2679,7 @@
       <c r="I100" s="27" t="n"/>
       <c r="J100" s="57" t="n"/>
     </row>
-    <row r="101" ht="20" customHeight="1" s="6">
+    <row r="101" ht="18" customHeight="1" s="6">
       <c r="A101" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -2711,7 +2711,7 @@
       <c r="I102" s="27" t="n"/>
       <c r="J102" s="57" t="n"/>
     </row>
-    <row r="103" ht="20" customHeight="1" s="6">
+    <row r="103" ht="18" customHeight="1" s="6">
       <c r="A103" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -2727,7 +2727,7 @@
       <c r="I103" s="27" t="n"/>
       <c r="J103" s="57" t="n"/>
     </row>
-    <row r="104" ht="20" customHeight="1" s="6">
+    <row r="104" ht="18" customHeight="1" s="6">
       <c r="A104" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -2743,7 +2743,7 @@
       <c r="I104" s="27" t="n"/>
       <c r="J104" s="57" t="n"/>
     </row>
-    <row r="105" ht="20" customHeight="1" s="6">
+    <row r="105" ht="18" customHeight="1" s="6">
       <c r="A105" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -2759,7 +2759,7 @@
       <c r="I105" s="27" t="n"/>
       <c r="J105" s="57" t="n"/>
     </row>
-    <row r="106" ht="20" customHeight="1" s="6">
+    <row r="106" ht="18" customHeight="1" s="6">
       <c r="A106" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -2836,7 +2836,7 @@
       <c r="I110" s="27" t="n"/>
       <c r="J110" s="57" t="n"/>
     </row>
-    <row r="111" ht="20" customHeight="1" s="6">
+    <row r="111" ht="18" customHeight="1" s="6">
       <c r="A111" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -2852,7 +2852,7 @@
       <c r="I111" s="27" t="n"/>
       <c r="J111" s="57" t="n"/>
     </row>
-    <row r="112" ht="20" customHeight="1" s="6">
+    <row r="112" ht="18" customHeight="1" s="6">
       <c r="A112" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -2884,7 +2884,7 @@
       <c r="I113" s="27" t="n"/>
       <c r="J113" s="57" t="n"/>
     </row>
-    <row r="114" ht="20" customHeight="1" s="6">
+    <row r="114" ht="18" customHeight="1" s="6">
       <c r="A114" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -2900,7 +2900,7 @@
       <c r="I114" s="27" t="n"/>
       <c r="J114" s="57" t="n"/>
     </row>
-    <row r="115" ht="20" customHeight="1" s="6">
+    <row r="115" ht="18" customHeight="1" s="6">
       <c r="A115" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -2916,7 +2916,7 @@
       <c r="I115" s="27" t="n"/>
       <c r="J115" s="57" t="n"/>
     </row>
-    <row r="116" ht="20" customHeight="1" s="6">
+    <row r="116" ht="18" customHeight="1" s="6">
       <c r="A116" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -2948,7 +2948,7 @@
       <c r="I117" s="27" t="n"/>
       <c r="J117" s="57" t="n"/>
     </row>
-    <row r="118" ht="20" customHeight="1" s="6">
+    <row r="118" ht="18" customHeight="1" s="6">
       <c r="A118" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -2964,7 +2964,7 @@
       <c r="I118" s="27" t="n"/>
       <c r="J118" s="57" t="n"/>
     </row>
-    <row r="119" ht="20" customHeight="1" s="6">
+    <row r="119" ht="18" customHeight="1" s="6">
       <c r="A119" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -2996,7 +2996,7 @@
       <c r="I120" s="27" t="n"/>
       <c r="J120" s="57" t="n"/>
     </row>
-    <row r="121" ht="20" customHeight="1" s="6">
+    <row r="121" ht="18" customHeight="1" s="6">
       <c r="A121" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -3012,7 +3012,7 @@
       <c r="I121" s="27" t="n"/>
       <c r="J121" s="57" t="n"/>
     </row>
-    <row r="122" ht="20" customHeight="1" s="6">
+    <row r="122" ht="18" customHeight="1" s="6">
       <c r="A122" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -3044,7 +3044,7 @@
       <c r="I123" s="27" t="n"/>
       <c r="J123" s="57" t="n"/>
     </row>
-    <row r="124" ht="20" customHeight="1" s="6">
+    <row r="124" ht="18" customHeight="1" s="6">
       <c r="A124" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -3060,7 +3060,7 @@
       <c r="I124" s="27" t="n"/>
       <c r="J124" s="57" t="n"/>
     </row>
-    <row r="125" ht="20" customHeight="1" s="6">
+    <row r="125" ht="18" customHeight="1" s="6">
       <c r="A125" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -3076,7 +3076,7 @@
       <c r="I125" s="27" t="n"/>
       <c r="J125" s="57" t="n"/>
     </row>
-    <row r="126" ht="20" customHeight="1" s="6">
+    <row r="126" ht="18" customHeight="1" s="6">
       <c r="A126" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -3092,7 +3092,7 @@
       <c r="I126" s="27" t="n"/>
       <c r="J126" s="57" t="n"/>
     </row>
-    <row r="127" ht="20" customHeight="1" s="6">
+    <row r="127" ht="18" customHeight="1" s="6">
       <c r="A127" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -3169,7 +3169,7 @@
       <c r="I131" s="27" t="n"/>
       <c r="J131" s="57" t="n"/>
     </row>
-    <row r="132" ht="20" customHeight="1" s="6">
+    <row r="132" ht="18" customHeight="1" s="6">
       <c r="A132" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -3185,7 +3185,7 @@
       <c r="I132" s="27" t="n"/>
       <c r="J132" s="57" t="n"/>
     </row>
-    <row r="133" ht="20" customHeight="1" s="6">
+    <row r="133" ht="18" customHeight="1" s="6">
       <c r="A133" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -3217,7 +3217,7 @@
       <c r="I134" s="27" t="n"/>
       <c r="J134" s="57" t="n"/>
     </row>
-    <row r="135" ht="20" customHeight="1" s="6">
+    <row r="135" ht="18" customHeight="1" s="6">
       <c r="A135" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -3233,7 +3233,7 @@
       <c r="I135" s="27" t="n"/>
       <c r="J135" s="57" t="n"/>
     </row>
-    <row r="136" ht="20" customHeight="1" s="6">
+    <row r="136" ht="18" customHeight="1" s="6">
       <c r="A136" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -3249,7 +3249,7 @@
       <c r="I136" s="27" t="n"/>
       <c r="J136" s="57" t="n"/>
     </row>
-    <row r="137" ht="20" customHeight="1" s="6">
+    <row r="137" ht="18" customHeight="1" s="6">
       <c r="A137" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -3281,7 +3281,7 @@
       <c r="I138" s="27" t="n"/>
       <c r="J138" s="57" t="n"/>
     </row>
-    <row r="139" ht="20" customHeight="1" s="6">
+    <row r="139" ht="18" customHeight="1" s="6">
       <c r="A139" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -3297,7 +3297,7 @@
       <c r="I139" s="27" t="n"/>
       <c r="J139" s="57" t="n"/>
     </row>
-    <row r="140" ht="20" customHeight="1" s="6">
+    <row r="140" ht="18" customHeight="1" s="6">
       <c r="A140" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -3329,7 +3329,7 @@
       <c r="I141" s="27" t="n"/>
       <c r="J141" s="57" t="n"/>
     </row>
-    <row r="142" ht="20" customHeight="1" s="6">
+    <row r="142" ht="18" customHeight="1" s="6">
       <c r="A142" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -3345,7 +3345,7 @@
       <c r="I142" s="27" t="n"/>
       <c r="J142" s="57" t="n"/>
     </row>
-    <row r="143" ht="20" customHeight="1" s="6">
+    <row r="143" ht="18" customHeight="1" s="6">
       <c r="A143" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -3377,7 +3377,7 @@
       <c r="I144" s="27" t="n"/>
       <c r="J144" s="57" t="n"/>
     </row>
-    <row r="145" ht="20" customHeight="1" s="6">
+    <row r="145" ht="18" customHeight="1" s="6">
       <c r="A145" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -3393,7 +3393,7 @@
       <c r="I145" s="27" t="n"/>
       <c r="J145" s="57" t="n"/>
     </row>
-    <row r="146" ht="20" customHeight="1" s="6">
+    <row r="146" ht="18" customHeight="1" s="6">
       <c r="A146" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -3409,7 +3409,7 @@
       <c r="I146" s="27" t="n"/>
       <c r="J146" s="57" t="n"/>
     </row>
-    <row r="147" ht="20" customHeight="1" s="6">
+    <row r="147" ht="18" customHeight="1" s="6">
       <c r="A147" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -3425,7 +3425,7 @@
       <c r="I147" s="27" t="n"/>
       <c r="J147" s="57" t="n"/>
     </row>
-    <row r="148" ht="20" customHeight="1" s="6">
+    <row r="148" ht="18" customHeight="1" s="6">
       <c r="A148" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -3502,7 +3502,7 @@
       <c r="I152" s="27" t="n"/>
       <c r="J152" s="57" t="n"/>
     </row>
-    <row r="153" ht="20" customHeight="1" s="6">
+    <row r="153" ht="18" customHeight="1" s="6">
       <c r="A153" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -3518,7 +3518,7 @@
       <c r="I153" s="27" t="n"/>
       <c r="J153" s="57" t="n"/>
     </row>
-    <row r="154" ht="20" customHeight="1" s="6">
+    <row r="154" ht="18" customHeight="1" s="6">
       <c r="A154" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -3550,7 +3550,7 @@
       <c r="I155" s="27" t="n"/>
       <c r="J155" s="57" t="n"/>
     </row>
-    <row r="156" ht="20" customHeight="1" s="6">
+    <row r="156" ht="18" customHeight="1" s="6">
       <c r="A156" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -3566,7 +3566,7 @@
       <c r="I156" s="27" t="n"/>
       <c r="J156" s="57" t="n"/>
     </row>
-    <row r="157" ht="20" customHeight="1" s="6">
+    <row r="157" ht="18" customHeight="1" s="6">
       <c r="A157" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -3582,7 +3582,7 @@
       <c r="I157" s="27" t="n"/>
       <c r="J157" s="57" t="n"/>
     </row>
-    <row r="158" ht="20" customHeight="1" s="6">
+    <row r="158" ht="18" customHeight="1" s="6">
       <c r="A158" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -3614,7 +3614,7 @@
       <c r="I159" s="27" t="n"/>
       <c r="J159" s="57" t="n"/>
     </row>
-    <row r="160" ht="20" customHeight="1" s="6">
+    <row r="160" ht="18" customHeight="1" s="6">
       <c r="A160" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -3630,7 +3630,7 @@
       <c r="I160" s="27" t="n"/>
       <c r="J160" s="57" t="n"/>
     </row>
-    <row r="161" ht="20" customHeight="1" s="6">
+    <row r="161" ht="18" customHeight="1" s="6">
       <c r="A161" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -3662,7 +3662,7 @@
       <c r="I162" s="27" t="n"/>
       <c r="J162" s="57" t="n"/>
     </row>
-    <row r="163" ht="20" customHeight="1" s="6">
+    <row r="163" ht="18" customHeight="1" s="6">
       <c r="A163" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -3678,7 +3678,7 @@
       <c r="I163" s="27" t="n"/>
       <c r="J163" s="57" t="n"/>
     </row>
-    <row r="164" ht="20" customHeight="1" s="6">
+    <row r="164" ht="18" customHeight="1" s="6">
       <c r="A164" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -3710,7 +3710,7 @@
       <c r="I165" s="27" t="n"/>
       <c r="J165" s="57" t="n"/>
     </row>
-    <row r="166" ht="20" customHeight="1" s="6">
+    <row r="166" ht="18" customHeight="1" s="6">
       <c r="A166" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -3726,7 +3726,7 @@
       <c r="I166" s="27" t="n"/>
       <c r="J166" s="57" t="n"/>
     </row>
-    <row r="167" ht="20" customHeight="1" s="6">
+    <row r="167" ht="18" customHeight="1" s="6">
       <c r="A167" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -3742,7 +3742,7 @@
       <c r="I167" s="27" t="n"/>
       <c r="J167" s="57" t="n"/>
     </row>
-    <row r="168" ht="20" customHeight="1" s="6">
+    <row r="168" ht="18" customHeight="1" s="6">
       <c r="A168" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -3758,7 +3758,7 @@
       <c r="I168" s="27" t="n"/>
       <c r="J168" s="57" t="n"/>
     </row>
-    <row r="169" ht="20" customHeight="1" s="6">
+    <row r="169" ht="18" customHeight="1" s="6">
       <c r="A169" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -3835,7 +3835,7 @@
       <c r="I173" s="27" t="n"/>
       <c r="J173" s="57" t="n"/>
     </row>
-    <row r="174" ht="20" customHeight="1" s="6">
+    <row r="174" ht="18" customHeight="1" s="6">
       <c r="A174" s="11" t="inlineStr">
         <is>
           <t>回答（can）：</t>
@@ -3851,7 +3851,7 @@
       <c r="I174" s="27" t="n"/>
       <c r="J174" s="57" t="n"/>
     </row>
-    <row r="175" ht="20" customHeight="1" s="6">
+    <row r="175" ht="18" customHeight="1" s="6">
       <c r="A175" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -3883,7 +3883,7 @@
       <c r="I176" s="27" t="n"/>
       <c r="J176" s="57" t="n"/>
     </row>
-    <row r="177" ht="20" customHeight="1" s="6">
+    <row r="177" ht="18" customHeight="1" s="6">
       <c r="A177" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -3899,7 +3899,7 @@
       <c r="I177" s="27" t="n"/>
       <c r="J177" s="57" t="n"/>
     </row>
-    <row r="178" ht="20" customHeight="1" s="6">
+    <row r="178" ht="18" customHeight="1" s="6">
       <c r="A178" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -3915,7 +3915,7 @@
       <c r="I178" s="27" t="n"/>
       <c r="J178" s="57" t="n"/>
     </row>
-    <row r="179" ht="20" customHeight="1" s="6">
+    <row r="179" ht="18" customHeight="1" s="6">
       <c r="A179" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ）：</t>
@@ -3947,7 +3947,7 @@
       <c r="I180" s="27" t="n"/>
       <c r="J180" s="57" t="n"/>
     </row>
-    <row r="181" ht="20" customHeight="1" s="6">
+    <row r="181" ht="18" customHeight="1" s="6">
       <c r="A181" s="11" t="inlineStr">
         <is>
           <t>回答（can疑問文）：</t>
@@ -3963,7 +3963,7 @@
       <c r="I181" s="27" t="n"/>
       <c r="J181" s="57" t="n"/>
     </row>
-    <row r="182" ht="20" customHeight="1" s="6">
+    <row r="182" ht="18" customHeight="1" s="6">
       <c r="A182" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ疑問文）：</t>
@@ -3995,7 +3995,7 @@
       <c r="I183" s="27" t="n"/>
       <c r="J183" s="57" t="n"/>
     </row>
-    <row r="184" ht="20" customHeight="1" s="6">
+    <row r="184" ht="18" customHeight="1" s="6">
       <c r="A184" s="11" t="inlineStr">
         <is>
           <t>回答（can返答）：</t>
@@ -4011,7 +4011,7 @@
       <c r="I184" s="27" t="n"/>
       <c r="J184" s="57" t="n"/>
     </row>
-    <row r="185" ht="20" customHeight="1" s="6">
+    <row r="185" ht="18" customHeight="1" s="6">
       <c r="A185" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ返答）：</t>
@@ -4043,7 +4043,7 @@
       <c r="I186" s="27" t="n"/>
       <c r="J186" s="57" t="n"/>
     </row>
-    <row r="187" ht="20" customHeight="1" s="6">
+    <row r="187" ht="18" customHeight="1" s="6">
       <c r="A187" s="11" t="inlineStr">
         <is>
           <t>回答（基本形）：</t>
@@ -4059,7 +4059,7 @@
       <c r="I187" s="27" t="n"/>
       <c r="J187" s="57" t="n"/>
     </row>
-    <row r="188" ht="20" customHeight="1" s="6">
+    <row r="188" ht="18" customHeight="1" s="6">
       <c r="A188" s="11" t="inlineStr">
         <is>
           <t>回答（短縮形）：</t>
@@ -4075,7 +4075,7 @@
       <c r="I188" s="27" t="n"/>
       <c r="J188" s="57" t="n"/>
     </row>
-    <row r="189" ht="20" customHeight="1" s="6">
+    <row r="189" ht="18" customHeight="1" s="6">
       <c r="A189" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ基本形）：</t>
@@ -4091,7 +4091,7 @@
       <c r="I189" s="27" t="n"/>
       <c r="J189" s="57" t="n"/>
     </row>
-    <row r="190" ht="20" customHeight="1" s="6">
+    <row r="190" ht="18" customHeight="1" s="6">
       <c r="A190" s="11" t="inlineStr">
         <is>
           <t>回答（言いかえ短縮形）：</t>
@@ -4136,8 +4136,8 @@
     <mergeCell ref="A93:J93"/>
     <mergeCell ref="A173:J173"/>
     <mergeCell ref="A130:J130"/>
+    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A83:J83"/>
-    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A34:J34"/>
     <mergeCell ref="A148:J148"/>
     <mergeCell ref="A157:J157"/>
@@ -4169,14 +4169,14 @@
     <mergeCell ref="A106:J106"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A81:J81"/>
     <mergeCell ref="A96:J96"/>
-    <mergeCell ref="A81:J81"/>
     <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A121:J121"/>
-    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A161:J161"/>
+    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A170:J170"/>
-    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A44:J44"/>
     <mergeCell ref="A31:J31"/>
     <mergeCell ref="A58:J58"/>
@@ -4219,11 +4219,11 @@
     <mergeCell ref="A122:J122"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="A125:J125"/>
+    <mergeCell ref="A190:J190"/>
     <mergeCell ref="A72:J72"/>
-    <mergeCell ref="A190:J190"/>
+    <mergeCell ref="A134:J134"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A112:J112"/>
-    <mergeCell ref="A134:J134"/>
     <mergeCell ref="A152:J152"/>
     <mergeCell ref="A167:J167"/>
     <mergeCell ref="A127:J127"/>
@@ -4235,9 +4235,9 @@
     <mergeCell ref="A64:J64"/>
     <mergeCell ref="A98:J98"/>
     <mergeCell ref="A191:J191"/>
+    <mergeCell ref="A169:J169"/>
     <mergeCell ref="A51:J51"/>
     <mergeCell ref="A107:J107"/>
-    <mergeCell ref="A169:J169"/>
     <mergeCell ref="A178:J178"/>
     <mergeCell ref="A79:J79"/>
     <mergeCell ref="A61:J61"/>
@@ -4267,13 +4267,13 @@
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="A188:J188"/>
     <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A131:J131"/>
     <mergeCell ref="A100:J100"/>
-    <mergeCell ref="A131:J131"/>
     <mergeCell ref="A126:J126"/>
+    <mergeCell ref="A140:J140"/>
+    <mergeCell ref="A53:J53"/>
     <mergeCell ref="A109:J109"/>
-    <mergeCell ref="A53:J53"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A140:J140"/>
     <mergeCell ref="A180:J180"/>
     <mergeCell ref="A129:J129"/>
     <mergeCell ref="A10:J10"/>
@@ -4314,8 +4314,8 @@
     <mergeCell ref="A185:J185"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
-  <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" verticalDpi="0"/>
+  <pageMargins left="0.4330708661417323" right="0.4330708661417323" top="0.5118110236220472" bottom="0.5118110236220472" header="0.1968503937007874" footer="0.1968503937007874"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" verticalDpi="0"/>
   <rowBreaks count="4" manualBreakCount="4">
     <brk id="44" min="0" max="16383" man="1"/>
     <brk id="86" min="0" max="16383" man="1"/>
@@ -4329,12 +4329,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:J191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
-    <col width="13" customWidth="1" style="6" min="1" max="1"/>
+    <col width="9.6328125" customWidth="1" style="6" min="1" max="1"/>
     <col width="13" customWidth="1" style="6" min="2" max="2"/>
     <col width="13" customWidth="1" style="6" min="3" max="3"/>
     <col width="13" customWidth="1" style="6" min="4" max="4"/>
@@ -4424,7 +4424,7 @@
       <c r="I5" s="27" t="n"/>
       <c r="J5" s="57" t="n"/>
     </row>
-    <row r="6" ht="20" customHeight="1" s="6">
+    <row r="6" ht="18" customHeight="1" s="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>正解（can）：I can play tennis.</t>
@@ -4440,7 +4440,7 @@
       <c r="I6" s="27" t="n"/>
       <c r="J6" s="57" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1" s="6">
+    <row r="7" ht="18" customHeight="1" s="6">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：I am able to play tennis.</t>
@@ -4472,7 +4472,7 @@
       <c r="I8" s="27" t="n"/>
       <c r="J8" s="57" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1" s="6">
+    <row r="9" ht="18" customHeight="1" s="6">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：I cannot play tennis.</t>
@@ -4488,7 +4488,7 @@
       <c r="I9" s="27" t="n"/>
       <c r="J9" s="57" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1" s="6">
+    <row r="10" ht="18" customHeight="1" s="6">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：I can't play tennis.</t>
@@ -4504,7 +4504,7 @@
       <c r="I10" s="27" t="n"/>
       <c r="J10" s="57" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1" s="6">
+    <row r="11" ht="18" customHeight="1" s="6">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：I am not able to play tennis.</t>
@@ -4536,7 +4536,7 @@
       <c r="I12" s="27" t="n"/>
       <c r="J12" s="57" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1" s="6">
+    <row r="13" ht="18" customHeight="1" s="6">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can I play tennis?</t>
@@ -4552,7 +4552,7 @@
       <c r="I13" s="27" t="n"/>
       <c r="J13" s="57" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1" s="6">
+    <row r="14" ht="18" customHeight="1" s="6">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Am I able to play tennis?</t>
@@ -4584,7 +4584,7 @@
       <c r="I15" s="27" t="n"/>
       <c r="J15" s="57" t="n"/>
     </row>
-    <row r="16" ht="20" customHeight="1" s="6">
+    <row r="16" ht="18" customHeight="1" s="6">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, you can.</t>
@@ -4600,7 +4600,7 @@
       <c r="I16" s="27" t="n"/>
       <c r="J16" s="57" t="n"/>
     </row>
-    <row r="17" ht="20" customHeight="1" s="6">
+    <row r="17" ht="18" customHeight="1" s="6">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, you are.</t>
@@ -4632,7 +4632,7 @@
       <c r="I18" s="27" t="n"/>
       <c r="J18" s="57" t="n"/>
     </row>
-    <row r="19" ht="20" customHeight="1" s="6">
+    <row r="19" ht="18" customHeight="1" s="6">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, you cannot.</t>
@@ -4648,7 +4648,7 @@
       <c r="I19" s="27" t="n"/>
       <c r="J19" s="57" t="n"/>
     </row>
-    <row r="20" ht="20" customHeight="1" s="6">
+    <row r="20" ht="18" customHeight="1" s="6">
       <c r="A20" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, you can't.</t>
@@ -4664,7 +4664,7 @@
       <c r="I20" s="27" t="n"/>
       <c r="J20" s="57" t="n"/>
     </row>
-    <row r="21" ht="20" customHeight="1" s="6">
+    <row r="21" ht="18" customHeight="1" s="6">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, you are not.</t>
@@ -4680,7 +4680,7 @@
       <c r="I21" s="27" t="n"/>
       <c r="J21" s="57" t="n"/>
     </row>
-    <row r="22" ht="20" customHeight="1" s="6">
+    <row r="22" ht="18" customHeight="1" s="6">
       <c r="A22" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, you aren't.</t>
@@ -4757,7 +4757,7 @@
       <c r="I26" s="27" t="n"/>
       <c r="J26" s="57" t="n"/>
     </row>
-    <row r="27" ht="20" customHeight="1" s="6">
+    <row r="27" ht="18" customHeight="1" s="6">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>正解（can）：You can play tennis.</t>
@@ -4773,7 +4773,7 @@
       <c r="I27" s="27" t="n"/>
       <c r="J27" s="57" t="n"/>
     </row>
-    <row r="28" ht="20" customHeight="1" s="6">
+    <row r="28" ht="18" customHeight="1" s="6">
       <c r="A28" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：You are able to play tennis.</t>
@@ -4805,7 +4805,7 @@
       <c r="I29" s="27" t="n"/>
       <c r="J29" s="57" t="n"/>
     </row>
-    <row r="30" ht="20" customHeight="1" s="6">
+    <row r="30" ht="18" customHeight="1" s="6">
       <c r="A30" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：You cannot play tennis.</t>
@@ -4821,7 +4821,7 @@
       <c r="I30" s="27" t="n"/>
       <c r="J30" s="57" t="n"/>
     </row>
-    <row r="31" ht="20" customHeight="1" s="6">
+    <row r="31" ht="18" customHeight="1" s="6">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：You can't play tennis.</t>
@@ -4837,7 +4837,7 @@
       <c r="I31" s="27" t="n"/>
       <c r="J31" s="57" t="n"/>
     </row>
-    <row r="32" ht="20" customHeight="1" s="6">
+    <row r="32" ht="18" customHeight="1" s="6">
       <c r="A32" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：You are not able to play tennis.</t>
@@ -4869,7 +4869,7 @@
       <c r="I33" s="27" t="n"/>
       <c r="J33" s="57" t="n"/>
     </row>
-    <row r="34" ht="20" customHeight="1" s="6">
+    <row r="34" ht="18" customHeight="1" s="6">
       <c r="A34" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can you play tennis?</t>
@@ -4885,7 +4885,7 @@
       <c r="I34" s="27" t="n"/>
       <c r="J34" s="57" t="n"/>
     </row>
-    <row r="35" ht="20" customHeight="1" s="6">
+    <row r="35" ht="18" customHeight="1" s="6">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Are you able to play tennis?</t>
@@ -4917,7 +4917,7 @@
       <c r="I36" s="27" t="n"/>
       <c r="J36" s="57" t="n"/>
     </row>
-    <row r="37" ht="20" customHeight="1" s="6">
+    <row r="37" ht="18" customHeight="1" s="6">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, I can.</t>
@@ -4933,7 +4933,7 @@
       <c r="I37" s="27" t="n"/>
       <c r="J37" s="57" t="n"/>
     </row>
-    <row r="38" ht="20" customHeight="1" s="6">
+    <row r="38" ht="18" customHeight="1" s="6">
       <c r="A38" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, I am.</t>
@@ -4965,7 +4965,7 @@
       <c r="I39" s="27" t="n"/>
       <c r="J39" s="57" t="n"/>
     </row>
-    <row r="40" ht="20" customHeight="1" s="6">
+    <row r="40" ht="18" customHeight="1" s="6">
       <c r="A40" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, I cannot.</t>
@@ -4981,7 +4981,7 @@
       <c r="I40" s="27" t="n"/>
       <c r="J40" s="57" t="n"/>
     </row>
-    <row r="41" ht="20" customHeight="1" s="6">
+    <row r="41" ht="18" customHeight="1" s="6">
       <c r="A41" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, I can't.</t>
@@ -4997,7 +4997,7 @@
       <c r="I41" s="27" t="n"/>
       <c r="J41" s="57" t="n"/>
     </row>
-    <row r="42" ht="20" customHeight="1" s="6">
+    <row r="42" ht="18" customHeight="1" s="6">
       <c r="A42" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, I am not.</t>
@@ -5013,7 +5013,7 @@
       <c r="I42" s="27" t="n"/>
       <c r="J42" s="57" t="n"/>
     </row>
-    <row r="43" ht="20" customHeight="1" s="6">
+    <row r="43" ht="18" customHeight="1" s="6">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, I'm not.</t>
@@ -5090,7 +5090,7 @@
       <c r="I47" s="27" t="n"/>
       <c r="J47" s="57" t="n"/>
     </row>
-    <row r="48" ht="20" customHeight="1" s="6">
+    <row r="48" ht="18" customHeight="1" s="6">
       <c r="A48" s="11" t="inlineStr">
         <is>
           <t>正解（can）：He can play tennis.</t>
@@ -5106,7 +5106,7 @@
       <c r="I48" s="27" t="n"/>
       <c r="J48" s="57" t="n"/>
     </row>
-    <row r="49" ht="20" customHeight="1" s="6">
+    <row r="49" ht="18" customHeight="1" s="6">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：He is able to play tennis.</t>
@@ -5138,7 +5138,7 @@
       <c r="I50" s="27" t="n"/>
       <c r="J50" s="57" t="n"/>
     </row>
-    <row r="51" ht="20" customHeight="1" s="6">
+    <row r="51" ht="18" customHeight="1" s="6">
       <c r="A51" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：He cannot play tennis.</t>
@@ -5154,7 +5154,7 @@
       <c r="I51" s="27" t="n"/>
       <c r="J51" s="57" t="n"/>
     </row>
-    <row r="52" ht="20" customHeight="1" s="6">
+    <row r="52" ht="18" customHeight="1" s="6">
       <c r="A52" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：He can't play tennis.</t>
@@ -5170,7 +5170,7 @@
       <c r="I52" s="27" t="n"/>
       <c r="J52" s="57" t="n"/>
     </row>
-    <row r="53" ht="20" customHeight="1" s="6">
+    <row r="53" ht="18" customHeight="1" s="6">
       <c r="A53" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：He is not able to play tennis.</t>
@@ -5202,7 +5202,7 @@
       <c r="I54" s="27" t="n"/>
       <c r="J54" s="57" t="n"/>
     </row>
-    <row r="55" ht="20" customHeight="1" s="6">
+    <row r="55" ht="18" customHeight="1" s="6">
       <c r="A55" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can he play tennis?</t>
@@ -5218,7 +5218,7 @@
       <c r="I55" s="27" t="n"/>
       <c r="J55" s="57" t="n"/>
     </row>
-    <row r="56" ht="20" customHeight="1" s="6">
+    <row r="56" ht="18" customHeight="1" s="6">
       <c r="A56" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Is he able to play tennis?</t>
@@ -5250,7 +5250,7 @@
       <c r="I57" s="27" t="n"/>
       <c r="J57" s="57" t="n"/>
     </row>
-    <row r="58" ht="20" customHeight="1" s="6">
+    <row r="58" ht="18" customHeight="1" s="6">
       <c r="A58" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, he can.</t>
@@ -5266,7 +5266,7 @@
       <c r="I58" s="27" t="n"/>
       <c r="J58" s="57" t="n"/>
     </row>
-    <row r="59" ht="20" customHeight="1" s="6">
+    <row r="59" ht="18" customHeight="1" s="6">
       <c r="A59" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, he is.</t>
@@ -5298,7 +5298,7 @@
       <c r="I60" s="27" t="n"/>
       <c r="J60" s="57" t="n"/>
     </row>
-    <row r="61" ht="20" customHeight="1" s="6">
+    <row r="61" ht="18" customHeight="1" s="6">
       <c r="A61" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, he cannot.</t>
@@ -5314,7 +5314,7 @@
       <c r="I61" s="27" t="n"/>
       <c r="J61" s="57" t="n"/>
     </row>
-    <row r="62" ht="20" customHeight="1" s="6">
+    <row r="62" ht="18" customHeight="1" s="6">
       <c r="A62" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, he can't.</t>
@@ -5330,7 +5330,7 @@
       <c r="I62" s="27" t="n"/>
       <c r="J62" s="57" t="n"/>
     </row>
-    <row r="63" ht="20" customHeight="1" s="6">
+    <row r="63" ht="18" customHeight="1" s="6">
       <c r="A63" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, he is not.</t>
@@ -5346,7 +5346,7 @@
       <c r="I63" s="27" t="n"/>
       <c r="J63" s="57" t="n"/>
     </row>
-    <row r="64" ht="20" customHeight="1" s="6">
+    <row r="64" ht="18" customHeight="1" s="6">
       <c r="A64" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, he isn't.</t>
@@ -5423,7 +5423,7 @@
       <c r="I68" s="27" t="n"/>
       <c r="J68" s="57" t="n"/>
     </row>
-    <row r="69" ht="20" customHeight="1" s="6">
+    <row r="69" ht="18" customHeight="1" s="6">
       <c r="A69" s="11" t="inlineStr">
         <is>
           <t>正解（can）：She can play tennis.</t>
@@ -5439,7 +5439,7 @@
       <c r="I69" s="27" t="n"/>
       <c r="J69" s="57" t="n"/>
     </row>
-    <row r="70" ht="20" customHeight="1" s="6">
+    <row r="70" ht="18" customHeight="1" s="6">
       <c r="A70" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：She is able to play tennis.</t>
@@ -5471,7 +5471,7 @@
       <c r="I71" s="27" t="n"/>
       <c r="J71" s="57" t="n"/>
     </row>
-    <row r="72" ht="20" customHeight="1" s="6">
+    <row r="72" ht="18" customHeight="1" s="6">
       <c r="A72" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：She cannot play tennis.</t>
@@ -5487,7 +5487,7 @@
       <c r="I72" s="27" t="n"/>
       <c r="J72" s="57" t="n"/>
     </row>
-    <row r="73" ht="20" customHeight="1" s="6">
+    <row r="73" ht="18" customHeight="1" s="6">
       <c r="A73" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：She can't play tennis.</t>
@@ -5503,7 +5503,7 @@
       <c r="I73" s="27" t="n"/>
       <c r="J73" s="57" t="n"/>
     </row>
-    <row r="74" ht="20" customHeight="1" s="6">
+    <row r="74" ht="18" customHeight="1" s="6">
       <c r="A74" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：She is not able to play tennis.</t>
@@ -5535,7 +5535,7 @@
       <c r="I75" s="27" t="n"/>
       <c r="J75" s="57" t="n"/>
     </row>
-    <row r="76" ht="20" customHeight="1" s="6">
+    <row r="76" ht="18" customHeight="1" s="6">
       <c r="A76" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can she play tennis?</t>
@@ -5551,7 +5551,7 @@
       <c r="I76" s="27" t="n"/>
       <c r="J76" s="57" t="n"/>
     </row>
-    <row r="77" ht="20" customHeight="1" s="6">
+    <row r="77" ht="18" customHeight="1" s="6">
       <c r="A77" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Is she able to play tennis?</t>
@@ -5583,7 +5583,7 @@
       <c r="I78" s="27" t="n"/>
       <c r="J78" s="57" t="n"/>
     </row>
-    <row r="79" ht="20" customHeight="1" s="6">
+    <row r="79" ht="18" customHeight="1" s="6">
       <c r="A79" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, she can.</t>
@@ -5599,7 +5599,7 @@
       <c r="I79" s="27" t="n"/>
       <c r="J79" s="57" t="n"/>
     </row>
-    <row r="80" ht="20" customHeight="1" s="6">
+    <row r="80" ht="18" customHeight="1" s="6">
       <c r="A80" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, she is.</t>
@@ -5631,7 +5631,7 @@
       <c r="I81" s="27" t="n"/>
       <c r="J81" s="57" t="n"/>
     </row>
-    <row r="82" ht="20" customHeight="1" s="6">
+    <row r="82" ht="18" customHeight="1" s="6">
       <c r="A82" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, she cannot.</t>
@@ -5647,7 +5647,7 @@
       <c r="I82" s="27" t="n"/>
       <c r="J82" s="57" t="n"/>
     </row>
-    <row r="83" ht="20" customHeight="1" s="6">
+    <row r="83" ht="18" customHeight="1" s="6">
       <c r="A83" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, she can't.</t>
@@ -5663,7 +5663,7 @@
       <c r="I83" s="27" t="n"/>
       <c r="J83" s="57" t="n"/>
     </row>
-    <row r="84" ht="20" customHeight="1" s="6">
+    <row r="84" ht="18" customHeight="1" s="6">
       <c r="A84" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, she is not.</t>
@@ -5679,7 +5679,7 @@
       <c r="I84" s="27" t="n"/>
       <c r="J84" s="57" t="n"/>
     </row>
-    <row r="85" ht="20" customHeight="1" s="6">
+    <row r="85" ht="18" customHeight="1" s="6">
       <c r="A85" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, she isn't.</t>
@@ -5757,7 +5757,7 @@
       <c r="I89" s="27" t="n"/>
       <c r="J89" s="57" t="n"/>
     </row>
-    <row r="90" ht="20" customHeight="1" s="6">
+    <row r="90" ht="18" customHeight="1" s="6">
       <c r="A90" s="11" t="inlineStr">
         <is>
           <t>正解（can）：We can play tennis.</t>
@@ -5773,7 +5773,7 @@
       <c r="I90" s="27" t="n"/>
       <c r="J90" s="57" t="n"/>
     </row>
-    <row r="91" ht="20" customHeight="1" s="6">
+    <row r="91" ht="18" customHeight="1" s="6">
       <c r="A91" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：We are able to play tennis.</t>
@@ -5805,7 +5805,7 @@
       <c r="I92" s="27" t="n"/>
       <c r="J92" s="57" t="n"/>
     </row>
-    <row r="93" ht="20" customHeight="1" s="6">
+    <row r="93" ht="18" customHeight="1" s="6">
       <c r="A93" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：We cannot play tennis.</t>
@@ -5821,7 +5821,7 @@
       <c r="I93" s="27" t="n"/>
       <c r="J93" s="57" t="n"/>
     </row>
-    <row r="94" ht="20" customHeight="1" s="6">
+    <row r="94" ht="18" customHeight="1" s="6">
       <c r="A94" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：We can't play tennis.</t>
@@ -5837,7 +5837,7 @@
       <c r="I94" s="27" t="n"/>
       <c r="J94" s="57" t="n"/>
     </row>
-    <row r="95" ht="20" customHeight="1" s="6">
+    <row r="95" ht="18" customHeight="1" s="6">
       <c r="A95" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：We are not able to play tennis.</t>
@@ -5869,7 +5869,7 @@
       <c r="I96" s="27" t="n"/>
       <c r="J96" s="57" t="n"/>
     </row>
-    <row r="97" ht="20" customHeight="1" s="6">
+    <row r="97" ht="18" customHeight="1" s="6">
       <c r="A97" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can we play tennis?</t>
@@ -5885,7 +5885,7 @@
       <c r="I97" s="27" t="n"/>
       <c r="J97" s="57" t="n"/>
     </row>
-    <row r="98" ht="20" customHeight="1" s="6">
+    <row r="98" ht="18" customHeight="1" s="6">
       <c r="A98" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Are we able to play tennis?</t>
@@ -5917,7 +5917,7 @@
       <c r="I99" s="27" t="n"/>
       <c r="J99" s="57" t="n"/>
     </row>
-    <row r="100" ht="20" customHeight="1" s="6">
+    <row r="100" ht="18" customHeight="1" s="6">
       <c r="A100" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, you can.</t>
@@ -5933,7 +5933,7 @@
       <c r="I100" s="27" t="n"/>
       <c r="J100" s="57" t="n"/>
     </row>
-    <row r="101" ht="20" customHeight="1" s="6">
+    <row r="101" ht="18" customHeight="1" s="6">
       <c r="A101" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, you are.</t>
@@ -5965,7 +5965,7 @@
       <c r="I102" s="27" t="n"/>
       <c r="J102" s="57" t="n"/>
     </row>
-    <row r="103" ht="20" customHeight="1" s="6">
+    <row r="103" ht="18" customHeight="1" s="6">
       <c r="A103" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, you cannot.</t>
@@ -5981,7 +5981,7 @@
       <c r="I103" s="27" t="n"/>
       <c r="J103" s="57" t="n"/>
     </row>
-    <row r="104" ht="20" customHeight="1" s="6">
+    <row r="104" ht="18" customHeight="1" s="6">
       <c r="A104" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, you can't.</t>
@@ -5997,7 +5997,7 @@
       <c r="I104" s="27" t="n"/>
       <c r="J104" s="57" t="n"/>
     </row>
-    <row r="105" ht="20" customHeight="1" s="6">
+    <row r="105" ht="18" customHeight="1" s="6">
       <c r="A105" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, you are not.</t>
@@ -6013,7 +6013,7 @@
       <c r="I105" s="27" t="n"/>
       <c r="J105" s="57" t="n"/>
     </row>
-    <row r="106" ht="20" customHeight="1" s="6">
+    <row r="106" ht="18" customHeight="1" s="6">
       <c r="A106" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, you aren't.</t>
@@ -6090,7 +6090,7 @@
       <c r="I110" s="27" t="n"/>
       <c r="J110" s="57" t="n"/>
     </row>
-    <row r="111" ht="20" customHeight="1" s="6">
+    <row r="111" ht="18" customHeight="1" s="6">
       <c r="A111" s="11" t="inlineStr">
         <is>
           <t>正解（can）：You can play tennis.</t>
@@ -6106,7 +6106,7 @@
       <c r="I111" s="27" t="n"/>
       <c r="J111" s="57" t="n"/>
     </row>
-    <row r="112" ht="20" customHeight="1" s="6">
+    <row r="112" ht="18" customHeight="1" s="6">
       <c r="A112" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：You are able to play tennis.</t>
@@ -6138,7 +6138,7 @@
       <c r="I113" s="27" t="n"/>
       <c r="J113" s="57" t="n"/>
     </row>
-    <row r="114" ht="20" customHeight="1" s="6">
+    <row r="114" ht="18" customHeight="1" s="6">
       <c r="A114" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：You cannot play tennis.</t>
@@ -6154,7 +6154,7 @@
       <c r="I114" s="27" t="n"/>
       <c r="J114" s="57" t="n"/>
     </row>
-    <row r="115" ht="20" customHeight="1" s="6">
+    <row r="115" ht="18" customHeight="1" s="6">
       <c r="A115" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：You can't play tennis.</t>
@@ -6170,7 +6170,7 @@
       <c r="I115" s="27" t="n"/>
       <c r="J115" s="57" t="n"/>
     </row>
-    <row r="116" ht="20" customHeight="1" s="6">
+    <row r="116" ht="18" customHeight="1" s="6">
       <c r="A116" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：You are not able to play tennis.</t>
@@ -6202,7 +6202,7 @@
       <c r="I117" s="27" t="n"/>
       <c r="J117" s="57" t="n"/>
     </row>
-    <row r="118" ht="20" customHeight="1" s="6">
+    <row r="118" ht="18" customHeight="1" s="6">
       <c r="A118" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can you play tennis?</t>
@@ -6218,7 +6218,7 @@
       <c r="I118" s="27" t="n"/>
       <c r="J118" s="57" t="n"/>
     </row>
-    <row r="119" ht="20" customHeight="1" s="6">
+    <row r="119" ht="18" customHeight="1" s="6">
       <c r="A119" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Are you able to play tennis?</t>
@@ -6250,7 +6250,7 @@
       <c r="I120" s="27" t="n"/>
       <c r="J120" s="57" t="n"/>
     </row>
-    <row r="121" ht="20" customHeight="1" s="6">
+    <row r="121" ht="18" customHeight="1" s="6">
       <c r="A121" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, we can.</t>
@@ -6266,7 +6266,7 @@
       <c r="I121" s="27" t="n"/>
       <c r="J121" s="57" t="n"/>
     </row>
-    <row r="122" ht="20" customHeight="1" s="6">
+    <row r="122" ht="18" customHeight="1" s="6">
       <c r="A122" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, we are.</t>
@@ -6298,7 +6298,7 @@
       <c r="I123" s="27" t="n"/>
       <c r="J123" s="57" t="n"/>
     </row>
-    <row r="124" ht="20" customHeight="1" s="6">
+    <row r="124" ht="18" customHeight="1" s="6">
       <c r="A124" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, we cannot.</t>
@@ -6314,7 +6314,7 @@
       <c r="I124" s="27" t="n"/>
       <c r="J124" s="57" t="n"/>
     </row>
-    <row r="125" ht="20" customHeight="1" s="6">
+    <row r="125" ht="18" customHeight="1" s="6">
       <c r="A125" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, we can't.</t>
@@ -6330,7 +6330,7 @@
       <c r="I125" s="27" t="n"/>
       <c r="J125" s="57" t="n"/>
     </row>
-    <row r="126" ht="20" customHeight="1" s="6">
+    <row r="126" ht="18" customHeight="1" s="6">
       <c r="A126" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, we are not.</t>
@@ -6346,7 +6346,7 @@
       <c r="I126" s="27" t="n"/>
       <c r="J126" s="57" t="n"/>
     </row>
-    <row r="127" ht="20" customHeight="1" s="6">
+    <row r="127" ht="18" customHeight="1" s="6">
       <c r="A127" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, we aren't.</t>
@@ -6423,7 +6423,7 @@
       <c r="I131" s="27" t="n"/>
       <c r="J131" s="57" t="n"/>
     </row>
-    <row r="132" ht="20" customHeight="1" s="6">
+    <row r="132" ht="18" customHeight="1" s="6">
       <c r="A132" s="11" t="inlineStr">
         <is>
           <t>正解（can）：They can play tennis.</t>
@@ -6439,7 +6439,7 @@
       <c r="I132" s="27" t="n"/>
       <c r="J132" s="57" t="n"/>
     </row>
-    <row r="133" ht="20" customHeight="1" s="6">
+    <row r="133" ht="18" customHeight="1" s="6">
       <c r="A133" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：They are able to play tennis.</t>
@@ -6471,7 +6471,7 @@
       <c r="I134" s="27" t="n"/>
       <c r="J134" s="57" t="n"/>
     </row>
-    <row r="135" ht="20" customHeight="1" s="6">
+    <row r="135" ht="18" customHeight="1" s="6">
       <c r="A135" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：They cannot play tennis.</t>
@@ -6487,7 +6487,7 @@
       <c r="I135" s="27" t="n"/>
       <c r="J135" s="57" t="n"/>
     </row>
-    <row r="136" ht="20" customHeight="1" s="6">
+    <row r="136" ht="18" customHeight="1" s="6">
       <c r="A136" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：They can't play tennis.</t>
@@ -6503,7 +6503,7 @@
       <c r="I136" s="27" t="n"/>
       <c r="J136" s="57" t="n"/>
     </row>
-    <row r="137" ht="20" customHeight="1" s="6">
+    <row r="137" ht="18" customHeight="1" s="6">
       <c r="A137" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：They are not able to play tennis.</t>
@@ -6535,7 +6535,7 @@
       <c r="I138" s="27" t="n"/>
       <c r="J138" s="57" t="n"/>
     </row>
-    <row r="139" ht="20" customHeight="1" s="6">
+    <row r="139" ht="18" customHeight="1" s="6">
       <c r="A139" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can they play tennis?</t>
@@ -6551,7 +6551,7 @@
       <c r="I139" s="27" t="n"/>
       <c r="J139" s="57" t="n"/>
     </row>
-    <row r="140" ht="20" customHeight="1" s="6">
+    <row r="140" ht="18" customHeight="1" s="6">
       <c r="A140" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Are they able to play tennis?</t>
@@ -6583,7 +6583,7 @@
       <c r="I141" s="27" t="n"/>
       <c r="J141" s="57" t="n"/>
     </row>
-    <row r="142" ht="20" customHeight="1" s="6">
+    <row r="142" ht="18" customHeight="1" s="6">
       <c r="A142" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, they can.</t>
@@ -6599,7 +6599,7 @@
       <c r="I142" s="27" t="n"/>
       <c r="J142" s="57" t="n"/>
     </row>
-    <row r="143" ht="20" customHeight="1" s="6">
+    <row r="143" ht="18" customHeight="1" s="6">
       <c r="A143" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, they are.</t>
@@ -6631,7 +6631,7 @@
       <c r="I144" s="27" t="n"/>
       <c r="J144" s="57" t="n"/>
     </row>
-    <row r="145" ht="20" customHeight="1" s="6">
+    <row r="145" ht="18" customHeight="1" s="6">
       <c r="A145" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, they cannot.</t>
@@ -6647,7 +6647,7 @@
       <c r="I145" s="27" t="n"/>
       <c r="J145" s="57" t="n"/>
     </row>
-    <row r="146" ht="20" customHeight="1" s="6">
+    <row r="146" ht="18" customHeight="1" s="6">
       <c r="A146" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, they can't.</t>
@@ -6663,7 +6663,7 @@
       <c r="I146" s="27" t="n"/>
       <c r="J146" s="57" t="n"/>
     </row>
-    <row r="147" ht="20" customHeight="1" s="6">
+    <row r="147" ht="18" customHeight="1" s="6">
       <c r="A147" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, they are not.</t>
@@ -6679,7 +6679,7 @@
       <c r="I147" s="27" t="n"/>
       <c r="J147" s="57" t="n"/>
     </row>
-    <row r="148" ht="20" customHeight="1" s="6">
+    <row r="148" ht="18" customHeight="1" s="6">
       <c r="A148" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, they aren't.</t>
@@ -6756,7 +6756,7 @@
       <c r="I152" s="27" t="n"/>
       <c r="J152" s="57" t="n"/>
     </row>
-    <row r="153" ht="20" customHeight="1" s="6">
+    <row r="153" ht="18" customHeight="1" s="6">
       <c r="A153" s="11" t="inlineStr">
         <is>
           <t>正解（can）：Ryoutarou can play tennis.</t>
@@ -6772,7 +6772,7 @@
       <c r="I153" s="27" t="n"/>
       <c r="J153" s="57" t="n"/>
     </row>
-    <row r="154" ht="20" customHeight="1" s="6">
+    <row r="154" ht="18" customHeight="1" s="6">
       <c r="A154" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：Ryoutarou is able to play tennis.</t>
@@ -6804,7 +6804,7 @@
       <c r="I155" s="27" t="n"/>
       <c r="J155" s="57" t="n"/>
     </row>
-    <row r="156" ht="20" customHeight="1" s="6">
+    <row r="156" ht="18" customHeight="1" s="6">
       <c r="A156" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：Ryoutarou cannot play tennis.</t>
@@ -6820,7 +6820,7 @@
       <c r="I156" s="27" t="n"/>
       <c r="J156" s="57" t="n"/>
     </row>
-    <row r="157" ht="20" customHeight="1" s="6">
+    <row r="157" ht="18" customHeight="1" s="6">
       <c r="A157" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：Ryoutarou can't play tennis.</t>
@@ -6836,7 +6836,7 @@
       <c r="I157" s="27" t="n"/>
       <c r="J157" s="57" t="n"/>
     </row>
-    <row r="158" ht="20" customHeight="1" s="6">
+    <row r="158" ht="18" customHeight="1" s="6">
       <c r="A158" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：Ryoutarou is not able to play tennis.</t>
@@ -6868,7 +6868,7 @@
       <c r="I159" s="27" t="n"/>
       <c r="J159" s="57" t="n"/>
     </row>
-    <row r="160" ht="20" customHeight="1" s="6">
+    <row r="160" ht="18" customHeight="1" s="6">
       <c r="A160" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can Ryoutarou play tennis?</t>
@@ -6884,7 +6884,7 @@
       <c r="I160" s="27" t="n"/>
       <c r="J160" s="57" t="n"/>
     </row>
-    <row r="161" ht="20" customHeight="1" s="6">
+    <row r="161" ht="18" customHeight="1" s="6">
       <c r="A161" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Is Ryoutarou able to play tennis?</t>
@@ -6916,7 +6916,7 @@
       <c r="I162" s="27" t="n"/>
       <c r="J162" s="57" t="n"/>
     </row>
-    <row r="163" ht="20" customHeight="1" s="6">
+    <row r="163" ht="18" customHeight="1" s="6">
       <c r="A163" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, he can.</t>
@@ -6932,7 +6932,7 @@
       <c r="I163" s="27" t="n"/>
       <c r="J163" s="57" t="n"/>
     </row>
-    <row r="164" ht="20" customHeight="1" s="6">
+    <row r="164" ht="18" customHeight="1" s="6">
       <c r="A164" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, he is.</t>
@@ -6964,7 +6964,7 @@
       <c r="I165" s="27" t="n"/>
       <c r="J165" s="57" t="n"/>
     </row>
-    <row r="166" ht="20" customHeight="1" s="6">
+    <row r="166" ht="18" customHeight="1" s="6">
       <c r="A166" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, he cannot.</t>
@@ -6980,7 +6980,7 @@
       <c r="I166" s="27" t="n"/>
       <c r="J166" s="57" t="n"/>
     </row>
-    <row r="167" ht="20" customHeight="1" s="6">
+    <row r="167" ht="18" customHeight="1" s="6">
       <c r="A167" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, he can't.</t>
@@ -6996,7 +6996,7 @@
       <c r="I167" s="27" t="n"/>
       <c r="J167" s="57" t="n"/>
     </row>
-    <row r="168" ht="20" customHeight="1" s="6">
+    <row r="168" ht="18" customHeight="1" s="6">
       <c r="A168" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, he is not.</t>
@@ -7012,7 +7012,7 @@
       <c r="I168" s="27" t="n"/>
       <c r="J168" s="57" t="n"/>
     </row>
-    <row r="169" ht="20" customHeight="1" s="6">
+    <row r="169" ht="18" customHeight="1" s="6">
       <c r="A169" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, he isn't.</t>
@@ -7089,7 +7089,7 @@
       <c r="I173" s="27" t="n"/>
       <c r="J173" s="57" t="n"/>
     </row>
-    <row r="174" ht="20" customHeight="1" s="6">
+    <row r="174" ht="18" customHeight="1" s="6">
       <c r="A174" s="11" t="inlineStr">
         <is>
           <t>正解（can）：Chisako can play tennis.</t>
@@ -7105,7 +7105,7 @@
       <c r="I174" s="27" t="n"/>
       <c r="J174" s="57" t="n"/>
     </row>
-    <row r="175" ht="20" customHeight="1" s="6">
+    <row r="175" ht="18" customHeight="1" s="6">
       <c r="A175" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：Chisako is able to play tennis.</t>
@@ -7137,7 +7137,7 @@
       <c r="I176" s="27" t="n"/>
       <c r="J176" s="57" t="n"/>
     </row>
-    <row r="177" ht="20" customHeight="1" s="6">
+    <row r="177" ht="18" customHeight="1" s="6">
       <c r="A177" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：Chisako cannot play tennis.</t>
@@ -7153,7 +7153,7 @@
       <c r="I177" s="27" t="n"/>
       <c r="J177" s="57" t="n"/>
     </row>
-    <row r="178" ht="20" customHeight="1" s="6">
+    <row r="178" ht="18" customHeight="1" s="6">
       <c r="A178" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：Chisako can't play tennis.</t>
@@ -7169,7 +7169,7 @@
       <c r="I178" s="27" t="n"/>
       <c r="J178" s="57" t="n"/>
     </row>
-    <row r="179" ht="20" customHeight="1" s="6">
+    <row r="179" ht="18" customHeight="1" s="6">
       <c r="A179" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ）：Chisako is not able to play tennis.</t>
@@ -7201,7 +7201,7 @@
       <c r="I180" s="27" t="n"/>
       <c r="J180" s="57" t="n"/>
     </row>
-    <row r="181" ht="20" customHeight="1" s="6">
+    <row r="181" ht="18" customHeight="1" s="6">
       <c r="A181" s="11" t="inlineStr">
         <is>
           <t>正解（can疑問文）：Can Chisako play tennis?</t>
@@ -7217,7 +7217,7 @@
       <c r="I181" s="27" t="n"/>
       <c r="J181" s="57" t="n"/>
     </row>
-    <row r="182" ht="20" customHeight="1" s="6">
+    <row r="182" ht="18" customHeight="1" s="6">
       <c r="A182" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ疑問文）：Is Chisako able to play tennis?</t>
@@ -7249,7 +7249,7 @@
       <c r="I183" s="27" t="n"/>
       <c r="J183" s="57" t="n"/>
     </row>
-    <row r="184" ht="20" customHeight="1" s="6">
+    <row r="184" ht="18" customHeight="1" s="6">
       <c r="A184" s="11" t="inlineStr">
         <is>
           <t>正解（can返答）：Yes, she can.</t>
@@ -7265,7 +7265,7 @@
       <c r="I184" s="27" t="n"/>
       <c r="J184" s="57" t="n"/>
     </row>
-    <row r="185" ht="20" customHeight="1" s="6">
+    <row r="185" ht="18" customHeight="1" s="6">
       <c r="A185" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ返答）：Yes, she is.</t>
@@ -7297,7 +7297,7 @@
       <c r="I186" s="27" t="n"/>
       <c r="J186" s="57" t="n"/>
     </row>
-    <row r="187" ht="20" customHeight="1" s="6">
+    <row r="187" ht="18" customHeight="1" s="6">
       <c r="A187" s="11" t="inlineStr">
         <is>
           <t>正解（基本形）：No, she cannot.</t>
@@ -7313,7 +7313,7 @@
       <c r="I187" s="27" t="n"/>
       <c r="J187" s="57" t="n"/>
     </row>
-    <row r="188" ht="20" customHeight="1" s="6">
+    <row r="188" ht="18" customHeight="1" s="6">
       <c r="A188" s="11" t="inlineStr">
         <is>
           <t>正解（短縮形）：No, she can't.</t>
@@ -7329,7 +7329,7 @@
       <c r="I188" s="27" t="n"/>
       <c r="J188" s="57" t="n"/>
     </row>
-    <row r="189" ht="20" customHeight="1" s="6">
+    <row r="189" ht="18" customHeight="1" s="6">
       <c r="A189" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ基本形）：No, she is not.</t>
@@ -7345,7 +7345,7 @@
       <c r="I189" s="27" t="n"/>
       <c r="J189" s="57" t="n"/>
     </row>
-    <row r="190" ht="20" customHeight="1" s="6">
+    <row r="190" ht="18" customHeight="1" s="6">
       <c r="A190" s="11" t="inlineStr">
         <is>
           <t>正解（言いかえ短縮形）：No, she isn't.</t>
@@ -7390,8 +7390,8 @@
     <mergeCell ref="A93:J93"/>
     <mergeCell ref="A173:J173"/>
     <mergeCell ref="A130:J130"/>
+    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A83:J83"/>
-    <mergeCell ref="A77:J77"/>
     <mergeCell ref="A34:J34"/>
     <mergeCell ref="A148:J148"/>
     <mergeCell ref="A157:J157"/>
@@ -7423,14 +7423,14 @@
     <mergeCell ref="A106:J106"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A81:J81"/>
     <mergeCell ref="A96:J96"/>
-    <mergeCell ref="A81:J81"/>
     <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A121:J121"/>
-    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A161:J161"/>
+    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A170:J170"/>
-    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A44:J44"/>
     <mergeCell ref="A31:J31"/>
     <mergeCell ref="A58:J58"/>
@@ -7473,11 +7473,11 @@
     <mergeCell ref="A122:J122"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="A125:J125"/>
+    <mergeCell ref="A190:J190"/>
     <mergeCell ref="A72:J72"/>
-    <mergeCell ref="A190:J190"/>
+    <mergeCell ref="A134:J134"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A112:J112"/>
-    <mergeCell ref="A134:J134"/>
     <mergeCell ref="A152:J152"/>
     <mergeCell ref="A167:J167"/>
     <mergeCell ref="A127:J127"/>
@@ -7489,9 +7489,9 @@
     <mergeCell ref="A64:J64"/>
     <mergeCell ref="A98:J98"/>
     <mergeCell ref="A191:J191"/>
+    <mergeCell ref="A169:J169"/>
     <mergeCell ref="A51:J51"/>
     <mergeCell ref="A107:J107"/>
-    <mergeCell ref="A169:J169"/>
     <mergeCell ref="A178:J178"/>
     <mergeCell ref="A79:J79"/>
     <mergeCell ref="A61:J61"/>
@@ -7521,13 +7521,13 @@
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="A188:J188"/>
     <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A131:J131"/>
     <mergeCell ref="A100:J100"/>
-    <mergeCell ref="A131:J131"/>
     <mergeCell ref="A126:J126"/>
+    <mergeCell ref="A140:J140"/>
+    <mergeCell ref="A53:J53"/>
     <mergeCell ref="A109:J109"/>
-    <mergeCell ref="A53:J53"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A140:J140"/>
     <mergeCell ref="A180:J180"/>
     <mergeCell ref="A129:J129"/>
     <mergeCell ref="A10:J10"/>
@@ -7568,8 +7568,8 @@
     <mergeCell ref="A185:J185"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
-  <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" verticalDpi="0"/>
+  <pageMargins left="0.4330708661417323" right="0.4330708661417323" top="0.5118110236220472" bottom="0.5118110236220472" header="0.1968503937007874" footer="0.1968503937007874"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" verticalDpi="0"/>
   <rowBreaks count="4" manualBreakCount="4">
     <brk id="44" min="0" max="16383" man="1"/>
     <brk id="86" min="0" max="16383" man="1"/>

</xml_diff>